<commit_message>
Ya entregué el asterisco
</commit_message>
<xml_diff>
--- a/Convoluciónes.xlsx
+++ b/Convoluciónes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\284\Desktop\Escuela\9no Semestre\Inteligencia Artificial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3175C6FA-34DF-48A6-8443-86B7D00826BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7E00929-45D6-452B-852C-292F4EC5D638}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C22957E8-8FCD-4F2E-90E1-3CD3928E7A2B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="25">
   <si>
     <t>Convolución 1</t>
   </si>
@@ -87,6 +87,30 @@
   </si>
   <si>
     <t>Convolución16</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>c3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>C6</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>c8</t>
+  </si>
+  <si>
+    <t>c9</t>
   </si>
 </sst>
 </file>
@@ -118,7 +142,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -242,6 +266,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -274,7 +304,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="12" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -346,7 +376,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -363,6 +392,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -698,14 +734,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BC98B396-EB36-4C61-A21E-152CA7B12277}">
-  <dimension ref="A1:O22"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="12.109375" customWidth="1"/>
     <col min="7" max="7" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="10">
         <v>0</v>
       </c>
@@ -725,7 +761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2" s="14">
         <v>0</v>
       </c>
@@ -745,7 +781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="21">
         <v>0</v>
       </c>
@@ -765,7 +801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="29">
         <v>0</v>
       </c>
@@ -794,23 +830,23 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A5" s="38">
-        <v>0</v>
-      </c>
-      <c r="B5" s="40">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5" s="37">
+        <v>0</v>
+      </c>
+      <c r="B5" s="39">
         <v>19</v>
       </c>
-      <c r="C5" s="43">
+      <c r="C5" s="42">
         <v>13</v>
       </c>
-      <c r="D5" s="44">
+      <c r="D5" s="43">
         <v>21</v>
       </c>
-      <c r="E5" s="44">
+      <c r="E5" s="43">
         <v>19</v>
       </c>
-      <c r="F5" s="44">
+      <c r="F5" s="43">
         <v>0</v>
       </c>
       <c r="H5" s="1">
@@ -823,23 +859,23 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="38">
-        <v>0</v>
-      </c>
-      <c r="B6" s="40">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6" s="37">
+        <v>0</v>
+      </c>
+      <c r="B6" s="39">
         <v>19</v>
       </c>
-      <c r="C6" s="43">
+      <c r="C6" s="42">
         <v>18</v>
       </c>
-      <c r="D6" s="44">
+      <c r="D6" s="43">
         <v>18</v>
       </c>
-      <c r="E6" s="44">
+      <c r="E6" s="43">
         <v>16</v>
       </c>
-      <c r="F6" s="44">
+      <c r="F6" s="43">
         <v>0</v>
       </c>
       <c r="H6" s="1">
@@ -852,23 +888,23 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A7" s="38">
-        <v>0</v>
-      </c>
-      <c r="B7" s="40">
-        <v>0</v>
-      </c>
-      <c r="C7" s="43">
-        <v>0</v>
-      </c>
-      <c r="D7" s="44">
-        <v>0</v>
-      </c>
-      <c r="E7" s="44">
-        <v>0</v>
-      </c>
-      <c r="F7" s="44">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7" s="37">
+        <v>0</v>
+      </c>
+      <c r="B7" s="39">
+        <v>0</v>
+      </c>
+      <c r="C7" s="42">
+        <v>0</v>
+      </c>
+      <c r="D7" s="43">
+        <v>0</v>
+      </c>
+      <c r="E7" s="43">
+        <v>0</v>
+      </c>
+      <c r="F7" s="43">
         <v>0</v>
       </c>
       <c r="H7" s="1">
@@ -881,7 +917,7 @@
         <v>0.1111111111111111</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>0</v>
       </c>
@@ -906,10 +942,10 @@
       <c r="H10" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="I10" s="39" t="s">
+      <c r="I10" s="38" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="39" t="s">
+      <c r="J10" s="38" t="s">
         <v>1</v>
       </c>
       <c r="K10" s="8">
@@ -929,7 +965,7 @@
         <v>26.888888888888889</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A1:C3)</f>
         <v>176</v>
@@ -987,7 +1023,7 @@
         <v>29.888888888888889</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
@@ -1012,10 +1048,10 @@
       <c r="H12" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="I12" s="41" t="s">
+      <c r="I12" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="41" t="s">
+      <c r="J12" s="40" t="s">
         <v>1</v>
       </c>
       <c r="K12" s="7">
@@ -1035,7 +1071,7 @@
         <v>22.111111111111111</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <f>SUM(B1:D3)</f>
         <v>248</v>
@@ -1093,7 +1129,7 @@
         <v>11.222222222222221</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>3</v>
       </c>
@@ -1118,10 +1154,10 @@
       <c r="H14" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="I14" s="42" t="s">
+      <c r="I14" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="J14" s="42" t="s">
+      <c r="J14" s="41" t="s">
         <v>1</v>
       </c>
       <c r="K14" s="7">
@@ -1141,7 +1177,7 @@
         <v>8.2222222222222214</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <f>SUM(C1:E3)</f>
         <v>392</v>
@@ -1182,13 +1218,8 @@
         <f>I15/9</f>
         <v>11.666666666666666</v>
       </c>
-      <c r="K15" s="37"/>
-      <c r="L15" s="37"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="37"/>
-      <c r="O15" s="37"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>4</v>
       </c>
@@ -1213,10 +1244,10 @@
       <c r="H16" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="I16" s="45" t="s">
+      <c r="I16" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="J16" s="45" t="s">
+      <c r="J16" s="44" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1262,8 +1293,207 @@
         <v>8.2222222222222214</v>
       </c>
     </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A20" s="46">
+        <v>0</v>
+      </c>
+      <c r="B20" s="46">
+        <v>0</v>
+      </c>
+      <c r="C20" s="46">
+        <v>0</v>
+      </c>
+      <c r="D20" s="46">
+        <v>0</v>
+      </c>
+      <c r="E20" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="46">
+        <v>0</v>
+      </c>
+      <c r="B21" s="45">
+        <v>3</v>
+      </c>
+      <c r="C21" s="45">
+        <v>2</v>
+      </c>
+      <c r="D21" s="45">
+        <v>5</v>
+      </c>
+      <c r="E21" s="46">
+        <v>0</v>
+      </c>
+    </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="J22" s="37"/>
+      <c r="A22" s="46">
+        <v>0</v>
+      </c>
+      <c r="B22" s="45">
+        <v>3</v>
+      </c>
+      <c r="C22" s="45">
+        <v>1</v>
+      </c>
+      <c r="D22" s="45">
+        <v>4</v>
+      </c>
+      <c r="E22" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="46">
+        <v>0</v>
+      </c>
+      <c r="B23" s="45">
+        <v>1</v>
+      </c>
+      <c r="C23" s="45">
+        <v>3</v>
+      </c>
+      <c r="D23" s="45">
+        <v>1</v>
+      </c>
+      <c r="E23" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="46">
+        <v>0</v>
+      </c>
+      <c r="B24" s="46">
+        <v>0</v>
+      </c>
+      <c r="C24" s="46">
+        <v>0</v>
+      </c>
+      <c r="D24" s="46">
+        <v>0</v>
+      </c>
+      <c r="E24" s="46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="H25" s="7">
+        <f>A27</f>
+        <v>9</v>
+      </c>
+      <c r="I25" s="7">
+        <f>A29</f>
+        <v>18</v>
+      </c>
+      <c r="J25" s="7">
+        <f>A31</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>0</v>
+      </c>
+      <c r="C26" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="7">
+        <f>C27</f>
+        <v>13</v>
+      </c>
+      <c r="I26" s="7">
+        <f>C29</f>
+        <v>23</v>
+      </c>
+      <c r="J26" s="7">
+        <f>C31</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <f>SUM(A20:C22)</f>
+        <v>9</v>
+      </c>
+      <c r="C27">
+        <f>SUM(A21:C23)</f>
+        <v>13</v>
+      </c>
+      <c r="E27">
+        <f>SUM(A22:C24)</f>
+        <v>8</v>
+      </c>
+      <c r="H27" s="7">
+        <f>E27</f>
+        <v>8</v>
+      </c>
+      <c r="I27" s="7">
+        <f>E29</f>
+        <v>13</v>
+      </c>
+      <c r="J27" s="7">
+        <f>E31</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>17</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="E28" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" s="47"/>
+      <c r="H28" s="47"/>
+      <c r="I28" s="47"/>
+      <c r="J28" s="47"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <f>SUM(B20:D22)</f>
+        <v>18</v>
+      </c>
+      <c r="C29">
+        <f>SUM(B21:D23)</f>
+        <v>23</v>
+      </c>
+      <c r="E29">
+        <f>SUM(B22:D24)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <f>SUM(C20:E22)</f>
+        <v>12</v>
+      </c>
+      <c r="C31">
+        <f>SUM(C21:E23)</f>
+        <v>16</v>
+      </c>
+      <c r="E31">
+        <f>SUM(C22:E24)</f>
+        <v>9</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>